<commit_message>
Modelos de planilha sem titular de exemplo
A prévia da importação recusa titular até a cifra por evento e os prazos do
jurídico (B.9); o modelo instalado precisa entrar sem erro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QKU6H2xGWvy1cxMQ5yybk3
</commit_message>
<xml_diff>
--- a/installer/modelos/modelo-cadastro-de-cartoes.xlsx
+++ b/installer/modelos/modelo-cadastro-de-cartoes.xlsx
@@ -25808,11 +25808,6 @@
           <t>SOCIAL</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Maria Exemplo</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>ATIVO</t>

</xml_diff>